<commit_message>
📦 NEW: monte carlo simulation
</commit_message>
<xml_diff>
--- a/Bingo_Musical_Boda_EstiCarles.xlsx
+++ b/Bingo_Musical_Boda_EstiCarles.xlsx
@@ -1,42 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\estra\Apps\bingo_musical\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7679C32F-241E-4F40-A088-50EBA58783C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Playlist" sheetId="2" r:id="rId1"/>
+    <sheet r:id="rId1" sheetId="1" name="Playlist"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="202">
   <si>
     <t>Nº</t>
   </si>
@@ -642,40 +620,33 @@
   </si>
   <si>
     <t>Despecha</t>
-  </si>
-  <si>
-    <t>Leyenda de categorias:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
+  <numFmts count="0"/>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FFffffff"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="12">
@@ -687,62 +658,52 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4472C4"/>
-        <bgColor rgb="FF666699"/>
+        <fgColor rgb="FF4472c4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBFBFBF"/>
-        <bgColor rgb="FFAAAAAA"/>
+        <fgColor rgb="FFbfbfbf"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFBDD7EE"/>
+        <fgColor rgb="FFd9d9d9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF4B183"/>
-        <bgColor rgb="FFFFD966"/>
+        <fgColor rgb="FFf4b183"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6E0B4"/>
-        <bgColor rgb="FFD9D9D9"/>
+        <fgColor rgb="FFc6e0b4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA9D18E"/>
-        <bgColor rgb="FFC6E0B4"/>
+        <fgColor rgb="FFa9d18e"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFD966"/>
-        <bgColor rgb="FFFFE699"/>
+        <fgColor rgb="FFffd966"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE699"/>
-        <bgColor rgb="FFFFD966"/>
+        <fgColor rgb="FFffe699"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF9DC3E6"/>
-        <bgColor rgb="FFBFBFBF"/>
+        <fgColor rgb="FF9dc3e6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFBDD7EE"/>
-        <bgColor rgb="FFD9D9D9"/>
+        <fgColor rgb="FFbdd7ee"/>
       </patternFill>
     </fill>
   </fills>
@@ -756,16 +717,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFAAAAAA"/>
+        <color rgb="FFaaaaaa"/>
       </left>
       <right style="thin">
-        <color rgb="FFAAAAAA"/>
+        <color rgb="FFaaaaaa"/>
       </right>
       <top style="thin">
-        <color rgb="FFAAAAAA"/>
+        <color rgb="FFaaaaaa"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFAAAAAA"/>
+        <color rgb="FFaaaaaa"/>
       </bottom>
       <diagonal/>
     </border>
@@ -773,155 +734,89 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+  <cellXfs count="25">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="11" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" builtinId="0" name="Normal"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFD9D9D9"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFBDD7EE"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFC6E0B4"/>
-      <rgbColor rgb="FFFFE699"/>
-      <rgbColor rgb="FF9DC3E6"/>
-      <rgbColor rgb="FFF4B183"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFD966"/>
-      <rgbColor rgb="FF4472C4"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FFA9D18E"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FFAAAAAA"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF2F5496"/>
-      <rgbColor rgb="FF333333"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -932,10 +827,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -973,128 +868,234 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme>
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="35000">
               <a:schemeClr val="phClr">
                 <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="9500"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot rev="0" lon="0" lat="0"/>
+            </a:camera>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="40000">
               <a:schemeClr val="phClr">
                 <a:tint val="45000"/>
                 <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
+                <a:tint val="80000"/>
+                <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1105,1410 +1106,1362 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D108"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="0"/>
+  </sheetPr>
+  <dimension ref="A1:D96"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="1" max="1" style="23" width="6.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="24" width="26.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="24" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="24" width="38.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A3" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A7" s="4">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A8" s="4">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A9" s="4">
         <v>8</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A10" s="4">
         <v>9</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A11" s="4">
         <v>10</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A12" s="4">
         <v>11</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="D12" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A13" s="4">
         <v>12</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="D13" s="6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A14" s="4">
         <v>13</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="D14" s="6" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A15" s="4">
         <v>14</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="D15" s="6" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A16" s="4">
         <v>15</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D16" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A17" s="4">
         <v>16</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A18" s="4">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="D18" s="6" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A19" s="4">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="D19" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A20" s="4">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="8" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A21" s="4">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A22" s="4">
         <v>21</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="8" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A23" s="4">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="8" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A24" s="4">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="8" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A25" s="4">
         <v>24</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="7" t="s">
+      <c r="C25" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="10" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A26" s="4">
         <v>25</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C26" s="7" t="s">
+      <c r="C26" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
+    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A27" s="4">
         <v>26</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C27" s="7" t="s">
+      <c r="C27" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D27" s="7" t="s">
+      <c r="D27" s="10" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A28" s="4">
         <v>27</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
+    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A29" s="4">
         <v>28</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C29" s="7" t="s">
+      <c r="C29" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D29" s="7" t="s">
+      <c r="D29" s="10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A30" s="4">
         <v>29</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D30" s="7" t="s">
+      <c r="D30" s="10" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
+    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A31" s="4">
         <v>30</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C31" s="7" t="s">
+      <c r="C31" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="7" t="s">
+      <c r="D31" s="10" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
+    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A32" s="4">
         <v>31</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="7" t="s">
+      <c r="D32" s="10" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
+    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A33" s="4">
         <v>32</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="D33" s="7" t="s">
+      <c r="D33" s="10" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
+    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A34" s="4">
         <v>33</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="D34" s="7" t="s">
+      <c r="D34" s="10" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
+    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A35" s="4">
         <v>34</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="D35" s="7" t="s">
+      <c r="D35" s="10" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A36" s="4">
         <v>35</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="C36" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="D36" s="7" t="s">
+      <c r="D36" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="2">
+    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A37" s="4">
         <v>36</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C37" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D37" s="7" t="s">
+      <c r="D37" s="10" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
+    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A38" s="4">
         <v>37</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C38" s="7" t="s">
+      <c r="C38" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="D38" s="7" t="s">
+      <c r="D38" s="10" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
+    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A39" s="4">
         <v>38</v>
       </c>
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C39" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D39" s="10" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
+    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A40" s="4">
         <v>39</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="7" t="s">
+      <c r="C40" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="D40" s="7" t="s">
+      <c r="D40" s="10" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A41" s="4">
         <v>40</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C41" s="7" t="s">
+      <c r="C41" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="D41" s="7" t="s">
+      <c r="D41" s="10" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
+    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A42" s="4">
         <v>41</v>
       </c>
-      <c r="B42" s="8" t="s">
+      <c r="B42" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="D42" s="9" t="s">
+      <c r="D42" s="12" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
+    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A43" s="4">
         <v>42</v>
       </c>
-      <c r="B43" s="8" t="s">
+      <c r="B43" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="D43" s="12" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
+    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A44" s="4">
         <v>43</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="D44" s="9" t="s">
+      <c r="D44" s="12" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
+    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A45" s="4">
         <v>44</v>
       </c>
-      <c r="B45" s="8" t="s">
+      <c r="B45" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="D45" s="9" t="s">
+      <c r="D45" s="12" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
+    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A46" s="4">
         <v>45</v>
       </c>
-      <c r="B46" s="8" t="s">
+      <c r="B46" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="D46" s="9" t="s">
+      <c r="D46" s="12" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="2">
+    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A47" s="4">
         <v>46</v>
       </c>
-      <c r="B47" s="8" t="s">
+      <c r="B47" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C47" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="D47" s="9" t="s">
+      <c r="D47" s="12" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="2">
+    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A48" s="4">
         <v>47</v>
       </c>
-      <c r="B48" s="8" t="s">
+      <c r="B48" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C48" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="D48" s="9" t="s">
+      <c r="D48" s="12" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
+    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A49" s="4">
         <v>48</v>
       </c>
-      <c r="B49" s="8" t="s">
+      <c r="B49" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="D49" s="9" t="s">
+      <c r="D49" s="12" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="2">
+    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A50" s="4">
         <v>49</v>
       </c>
-      <c r="B50" s="8" t="s">
+      <c r="B50" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="C50" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="D50" s="9" t="s">
+      <c r="D50" s="12" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="2">
+    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A51" s="4">
         <v>50</v>
       </c>
-      <c r="B51" s="10" t="s">
+      <c r="B51" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C51" s="11" t="s">
+      <c r="C51" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="D51" s="11" t="s">
+      <c r="D51" s="14" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="2">
+    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A52" s="4">
         <v>51</v>
       </c>
-      <c r="B52" s="10" t="s">
+      <c r="B52" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C52" s="11" t="s">
+      <c r="C52" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="D52" s="11" t="s">
+      <c r="D52" s="14" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="2">
+    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A53" s="4">
         <v>52</v>
       </c>
-      <c r="B53" s="10" t="s">
+      <c r="B53" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C53" s="11" t="s">
+      <c r="C53" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="D53" s="11" t="s">
+      <c r="D53" s="14" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="2">
+    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A54" s="4">
         <v>53</v>
       </c>
-      <c r="B54" s="10" t="s">
+      <c r="B54" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C54" s="11" t="s">
+      <c r="C54" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="D54" s="11" t="s">
+      <c r="D54" s="14" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="2">
+    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A55" s="4">
         <v>54</v>
       </c>
-      <c r="B55" s="10" t="s">
+      <c r="B55" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C55" s="11" t="s">
+      <c r="C55" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="D55" s="11" t="s">
+      <c r="D55" s="14" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="2">
+    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A56" s="4">
         <v>55</v>
       </c>
-      <c r="B56" s="10" t="s">
+      <c r="B56" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C56" s="11" t="s">
+      <c r="C56" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="D56" s="11" t="s">
+      <c r="D56" s="14" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="2">
+    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A57" s="4">
         <v>56</v>
       </c>
-      <c r="B57" s="10" t="s">
+      <c r="B57" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C57" s="11" t="s">
+      <c r="C57" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="D57" s="11" t="s">
+      <c r="D57" s="14" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="2">
+    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A58" s="4">
         <v>57</v>
       </c>
-      <c r="B58" s="10" t="s">
+      <c r="B58" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C58" s="11" t="s">
+      <c r="C58" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="D58" s="11" t="s">
+      <c r="D58" s="14" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="2">
+    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A59" s="4">
         <v>58</v>
       </c>
-      <c r="B59" s="10" t="s">
+      <c r="B59" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C59" s="11" t="s">
+      <c r="C59" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D59" s="11" t="s">
+      <c r="D59" s="14" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="2">
+    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A60" s="4">
         <v>59</v>
       </c>
-      <c r="B60" s="10" t="s">
+      <c r="B60" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="C60" s="11" t="s">
+      <c r="C60" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="D60" s="11" t="s">
+      <c r="D60" s="14" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="2">
+    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A61" s="4">
         <v>60</v>
       </c>
-      <c r="B61" s="12" t="s">
+      <c r="B61" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C61" s="13" t="s">
+      <c r="C61" s="16" t="s">
         <v>127</v>
       </c>
-      <c r="D61" s="13" t="s">
+      <c r="D61" s="16" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="2">
+    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A62" s="4">
         <v>61</v>
       </c>
-      <c r="B62" s="12" t="s">
+      <c r="B62" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C62" s="13" t="s">
+      <c r="C62" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="D62" s="13" t="s">
+      <c r="D62" s="16" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="2">
+    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A63" s="4">
         <v>62</v>
       </c>
-      <c r="B63" s="12" t="s">
+      <c r="B63" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C63" s="13" t="s">
+      <c r="C63" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="D63" s="13" t="s">
+      <c r="D63" s="16" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="2">
+    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A64" s="4">
         <v>63</v>
       </c>
-      <c r="B64" s="12" t="s">
+      <c r="B64" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C64" s="13" t="s">
+      <c r="C64" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="D64" s="13" t="s">
+      <c r="D64" s="16" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="2">
+    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A65" s="4">
         <v>64</v>
       </c>
-      <c r="B65" s="12" t="s">
+      <c r="B65" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C65" s="13" t="s">
+      <c r="C65" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="D65" s="13" t="s">
+      <c r="D65" s="16" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="2">
+    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A66" s="4">
         <v>65</v>
       </c>
-      <c r="B66" s="12" t="s">
+      <c r="B66" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C66" s="13" t="s">
+      <c r="C66" s="16" t="s">
         <v>137</v>
       </c>
-      <c r="D66" s="13" t="s">
+      <c r="D66" s="16" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="2">
+    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A67" s="4">
         <v>66</v>
       </c>
-      <c r="B67" s="12" t="s">
+      <c r="B67" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C67" s="13" t="s">
+      <c r="C67" s="16" t="s">
         <v>139</v>
       </c>
-      <c r="D67" s="13" t="s">
+      <c r="D67" s="16" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="2">
+    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A68" s="4">
         <v>67</v>
       </c>
-      <c r="B68" s="12" t="s">
+      <c r="B68" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C68" s="13" t="s">
+      <c r="C68" s="16" t="s">
         <v>141</v>
       </c>
-      <c r="D68" s="13" t="s">
+      <c r="D68" s="16" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="2">
+    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A69" s="4">
         <v>68</v>
       </c>
-      <c r="B69" s="12" t="s">
+      <c r="B69" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C69" s="13" t="s">
+      <c r="C69" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="D69" s="13" t="s">
+      <c r="D69" s="16" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="2">
+    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A70" s="4">
         <v>69</v>
       </c>
-      <c r="B70" s="12" t="s">
+      <c r="B70" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="C70" s="13" t="s">
+      <c r="C70" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="D70" s="13" t="s">
+      <c r="D70" s="16" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="2">
+    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A71" s="4">
         <v>70</v>
       </c>
-      <c r="B71" s="14" t="s">
+      <c r="B71" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C71" s="15" t="s">
+      <c r="C71" s="18" t="s">
         <v>148</v>
       </c>
-      <c r="D71" s="15" t="s">
+      <c r="D71" s="18" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="2">
+    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A72" s="4">
         <v>71</v>
       </c>
-      <c r="B72" s="14" t="s">
+      <c r="B72" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C72" s="15" t="s">
+      <c r="C72" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="D72" s="15" t="s">
+      <c r="D72" s="18" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="2">
+    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A73" s="4">
         <v>72</v>
       </c>
-      <c r="B73" s="14" t="s">
+      <c r="B73" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C73" s="15" t="s">
+      <c r="C73" s="18" t="s">
         <v>152</v>
       </c>
-      <c r="D73" s="15" t="s">
+      <c r="D73" s="18" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="2">
+    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A74" s="4">
         <v>73</v>
       </c>
-      <c r="B74" s="14" t="s">
+      <c r="B74" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C74" s="15" t="s">
+      <c r="C74" s="18" t="s">
         <v>154</v>
       </c>
-      <c r="D74" s="15" t="s">
+      <c r="D74" s="18" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="2">
+    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A75" s="4">
         <v>74</v>
       </c>
-      <c r="B75" s="14" t="s">
+      <c r="B75" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C75" s="15" t="s">
+      <c r="C75" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="D75" s="15" t="s">
+      <c r="D75" s="18" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="2">
+    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A76" s="4">
         <v>75</v>
       </c>
-      <c r="B76" s="14" t="s">
+      <c r="B76" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C76" s="15" t="s">
+      <c r="C76" s="18" t="s">
         <v>158</v>
       </c>
-      <c r="D76" s="15" t="s">
+      <c r="D76" s="18" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="2">
+    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A77" s="4">
         <v>76</v>
       </c>
-      <c r="B77" s="14" t="s">
+      <c r="B77" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C77" s="15" t="s">
+      <c r="C77" s="18" t="s">
         <v>160</v>
       </c>
-      <c r="D77" s="15" t="s">
+      <c r="D77" s="18" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="2">
+    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A78" s="4">
         <v>77</v>
       </c>
-      <c r="B78" s="14" t="s">
+      <c r="B78" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C78" s="15" t="s">
+      <c r="C78" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="D78" s="15" t="s">
+      <c r="D78" s="18" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="2">
+    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A79" s="4">
         <v>78</v>
       </c>
-      <c r="B79" s="14" t="s">
+      <c r="B79" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C79" s="15" t="s">
+      <c r="C79" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D79" s="15" t="s">
+      <c r="D79" s="18" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="2">
+    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A80" s="4">
         <v>79</v>
       </c>
-      <c r="B80" s="14" t="s">
+      <c r="B80" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C80" s="15" t="s">
+      <c r="C80" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="D80" s="15" t="s">
+      <c r="D80" s="18" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="2">
+    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A81" s="4">
         <v>80</v>
       </c>
-      <c r="B81" s="14" t="s">
+      <c r="B81" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C81" s="15" t="s">
+      <c r="C81" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="D81" s="15" t="s">
+      <c r="D81" s="18" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="2">
+    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A82" s="4">
         <v>81</v>
       </c>
-      <c r="B82" s="14" t="s">
+      <c r="B82" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C82" s="15" t="s">
+      <c r="C82" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="D82" s="15" t="s">
+      <c r="D82" s="18" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="2">
+    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A83" s="4">
         <v>82</v>
       </c>
-      <c r="B83" s="14" t="s">
+      <c r="B83" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="C83" s="15" t="s">
+      <c r="C83" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="D83" s="15" t="s">
+      <c r="D83" s="18" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="2">
+    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A84" s="4">
         <v>83</v>
       </c>
-      <c r="B84" s="16" t="s">
+      <c r="B84" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C84" s="17" t="s">
+      <c r="C84" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="D84" s="17" t="s">
+      <c r="D84" s="20" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="2">
+    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A85" s="4">
         <v>84</v>
       </c>
-      <c r="B85" s="16" t="s">
+      <c r="B85" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C85" s="17" t="s">
+      <c r="C85" s="20" t="s">
         <v>177</v>
       </c>
-      <c r="D85" s="17" t="s">
+      <c r="D85" s="20" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="2">
+    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A86" s="4">
         <v>85</v>
       </c>
-      <c r="B86" s="16" t="s">
+      <c r="B86" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C86" s="17" t="s">
+      <c r="C86" s="20" t="s">
         <v>179</v>
       </c>
-      <c r="D86" s="17" t="s">
+      <c r="D86" s="20" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="2">
+    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A87" s="4">
         <v>86</v>
       </c>
-      <c r="B87" s="16" t="s">
+      <c r="B87" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C87" s="17" t="s">
+      <c r="C87" s="20" t="s">
         <v>181</v>
       </c>
-      <c r="D87" s="17" t="s">
+      <c r="D87" s="20" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="2">
+    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A88" s="4">
         <v>87</v>
       </c>
-      <c r="B88" s="16" t="s">
+      <c r="B88" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C88" s="17" t="s">
+      <c r="C88" s="20" t="s">
         <v>183</v>
       </c>
-      <c r="D88" s="17" t="s">
+      <c r="D88" s="20" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="2">
+    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A89" s="4">
         <v>88</v>
       </c>
-      <c r="B89" s="16" t="s">
+      <c r="B89" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C89" s="17" t="s">
+      <c r="C89" s="20" t="s">
         <v>185</v>
       </c>
-      <c r="D89" s="17" t="s">
+      <c r="D89" s="20" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="2">
+    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A90" s="4">
         <v>89</v>
       </c>
-      <c r="B90" s="16"/>
-      <c r="C90" s="17" t="s">
+      <c r="B90" s="19"/>
+      <c r="C90" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="D90" s="17" t="s">
+      <c r="D90" s="20" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="2">
+    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A91" s="4">
         <v>90</v>
       </c>
-      <c r="B91" s="16" t="s">
+      <c r="B91" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C91" s="17" t="s">
+      <c r="C91" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="D91" s="17" t="s">
+      <c r="D91" s="20" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="2">
+    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A92" s="4">
         <v>91</v>
       </c>
-      <c r="B92" s="16" t="s">
+      <c r="B92" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C92" s="17" t="s">
+      <c r="C92" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="D92" s="17" t="s">
+      <c r="D92" s="20" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="2">
+    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A93" s="4">
         <v>92</v>
       </c>
-      <c r="B93" s="16" t="s">
+      <c r="B93" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="C93" s="17" t="s">
+      <c r="C93" s="20" t="s">
         <v>193</v>
       </c>
-      <c r="D93" s="17" t="s">
+      <c r="D93" s="20" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="2">
+    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A94" s="4">
         <v>93</v>
       </c>
-      <c r="B94" s="18" t="s">
+      <c r="B94" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="C94" s="19" t="s">
+      <c r="C94" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="D94" s="19" t="s">
+      <c r="D94" s="22" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="2">
+    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A95" s="4">
         <v>94</v>
       </c>
-      <c r="B95" s="18" t="s">
+      <c r="B95" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="C95" s="19" t="s">
+      <c r="C95" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="D95" s="19" t="s">
+      <c r="D95" s="22" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="2">
+    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75" customFormat="1" s="1">
+      <c r="A96" s="4">
         <v>95</v>
       </c>
-      <c r="B96" s="18" t="s">
+      <c r="B96" s="21" t="s">
         <v>195</v>
       </c>
-      <c r="C96" s="19" t="s">
+      <c r="C96" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="D96" s="19" t="s">
+      <c r="D96" s="22" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99" s="20" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" s="21" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" s="22" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A102" s="23" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A103" s="24" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A104" s="25" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A105" s="26" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A106" s="27" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A107" s="28" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A108" s="29" t="s">
-        <v>195</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>